<commit_message>
Final revision sync: align source data and supplementary analyses
</commit_message>
<xml_diff>
--- a/data_public/supplementary_tables/Table S6.xlsx
+++ b/data_public/supplementary_tables/Table S6.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section_Donor_Map" sheetId="1" r:id="R96a4917ba2854c09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spatial_Score_Definitions" sheetId="2" r:id="R1b2c4af8dd2d4819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spatial_Method_Parameters" sheetId="3" r:id="R2cac9a9bf22142b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section_Donor_Map" sheetId="1" r:id="Rbf54da2ba93e4353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spatial_Score_Definitions" sheetId="2" r:id="R9a92f28360584dd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spatial_Method_Parameters" sheetId="3" r:id="R05c32f4946dc4706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Donor_Level_Spatial_Endpoints" sheetId="4" r:id="R6ecc4831e1754c87"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0.0000000000"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,8 +54,12 @@
       <x:color rgb="FF243A52"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +76,11 @@
         <x:fgColor rgb="FFF2F4F7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -78,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -114,6 +124,21 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -645,7 +670,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f8927cd2d0d465d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99b9721b323247cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50548,7 +50573,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b13ab3a68aa41fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea51cea537674ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50780,7 +50805,384 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0e6e48d7e144984"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a6686652381422a"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="18" t="str">
+        <x:v>record_type</x:v>
+      </x:c>
+      <x:c r="B1" s="18" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="C1" s="18" t="str">
+        <x:v>sample_id</x:v>
+      </x:c>
+      <x:c r="D1" s="18" t="str">
+        <x:v>condition</x:v>
+      </x:c>
+      <x:c r="E1" s="18" t="str">
+        <x:v>GART_undetected_mean_program_score</x:v>
+      </x:c>
+      <x:c r="F1" s="18" t="str">
+        <x:v>GART_detected_mean_program_score</x:v>
+      </x:c>
+      <x:c r="G1" s="18" t="str">
+        <x:v>within_donor_difference</x:v>
+      </x:c>
+      <x:c r="H1" s="18" t="str">
+        <x:v>GART_undetected_spots</x:v>
+      </x:c>
+      <x:c r="I1" s="18" t="str">
+        <x:v>GART_detected_spots</x:v>
+      </x:c>
+      <x:c r="J1" s="18" t="str">
+        <x:v>mean_difference</x:v>
+      </x:c>
+      <x:c r="K1" s="18" t="str">
+        <x:v>CI_lower</x:v>
+      </x:c>
+      <x:c r="L1" s="18" t="str">
+        <x:v>CI_upper</x:v>
+      </x:c>
+      <x:c r="M1" s="18" t="str">
+        <x:v>exact_paired_sign_flip_P</x:v>
+      </x:c>
+      <x:c r="N1" s="18" t="str">
+        <x:v>positive_donors</x:v>
+      </x:c>
+      <x:c r="O1" s="18" t="str">
+        <x:v>n_donors</x:v>
+      </x:c>
+      <x:c r="P1" s="18" t="str">
+        <x:v>biological_replicate_note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B2" s="21" t="str">
+        <x:v>GI 6925</x:v>
+      </x:c>
+      <x:c r="C2" s="21" t="str">
+        <x:v>HC1</x:v>
+      </x:c>
+      <x:c r="D2" s="21" t="str">
+        <x:v>HC</x:v>
+      </x:c>
+      <x:c r="E2" s="21" t="n">
+        <x:v>0.5415172193429265</x:v>
+      </x:c>
+      <x:c r="F2" s="21" t="n">
+        <x:v>0.561410524986885</x:v>
+      </x:c>
+      <x:c r="G2" s="21" t="n">
+        <x:v>0.019893305643958525</x:v>
+      </x:c>
+      <x:c r="H2" s="21" t="n">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="I2" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J2" s="21"/>
+      <x:c r="K2" s="21"/>
+      <x:c r="L2" s="21"/>
+      <x:c r="M2" s="21"/>
+      <x:c r="N2" s="21"/>
+      <x:c r="O2" s="21"/>
+      <x:c r="P2" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B3" s="21" t="str">
+        <x:v>TIP 517</x:v>
+      </x:c>
+      <x:c r="C3" s="21" t="str">
+        <x:v>HC2</x:v>
+      </x:c>
+      <x:c r="D3" s="21" t="str">
+        <x:v>HC</x:v>
+      </x:c>
+      <x:c r="E3" s="21" t="n">
+        <x:v>0.6474167083423538</x:v>
+      </x:c>
+      <x:c r="F3" s="21" t="n">
+        <x:v>0.6797836826100317</x:v>
+      </x:c>
+      <x:c r="G3" s="21" t="n">
+        <x:v>0.032366974267677984</x:v>
+      </x:c>
+      <x:c r="H3" s="21" t="n">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="I3" s="21" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="J3" s="21"/>
+      <x:c r="K3" s="21"/>
+      <x:c r="L3" s="21"/>
+      <x:c r="M3" s="21"/>
+      <x:c r="N3" s="21"/>
+      <x:c r="O3" s="21"/>
+      <x:c r="P3" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="str">
+        <x:v>GI 6266</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>UC1</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>UC</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="n">
+        <x:v>0.5377122003704765</x:v>
+      </x:c>
+      <x:c r="F4" s="21" t="n">
+        <x:v>0.555571073291486</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="n">
+        <x:v>0.017858872921009517</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J4" s="21"/>
+      <x:c r="K4" s="21"/>
+      <x:c r="L4" s="21"/>
+      <x:c r="M4" s="21"/>
+      <x:c r="N4" s="21"/>
+      <x:c r="O4" s="21"/>
+      <x:c r="P4" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B5" s="21" t="str">
+        <x:v>GI 6264</x:v>
+      </x:c>
+      <x:c r="C5" s="21" t="str">
+        <x:v>UC2</x:v>
+      </x:c>
+      <x:c r="D5" s="21" t="str">
+        <x:v>UC</x:v>
+      </x:c>
+      <x:c r="E5" s="21" t="n">
+        <x:v>0.5511906556539987</x:v>
+      </x:c>
+      <x:c r="F5" s="21" t="n">
+        <x:v>0.5554316503909263</x:v>
+      </x:c>
+      <x:c r="G5" s="21" t="n">
+        <x:v>0.004240994736927628</x:v>
+      </x:c>
+      <x:c r="H5" s="21" t="n">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="I5" s="21" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="J5" s="21"/>
+      <x:c r="K5" s="21"/>
+      <x:c r="L5" s="21"/>
+      <x:c r="M5" s="21"/>
+      <x:c r="N5" s="21"/>
+      <x:c r="O5" s="21"/>
+      <x:c r="P5" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B6" s="21" t="str">
+        <x:v>GI 6658</x:v>
+      </x:c>
+      <x:c r="C6" s="21" t="str">
+        <x:v>UC3</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="str">
+        <x:v>UC</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="n">
+        <x:v>0.5466748938671503</x:v>
+      </x:c>
+      <x:c r="F6" s="21" t="n">
+        <x:v>0.5606921101851656</x:v>
+      </x:c>
+      <x:c r="G6" s="21" t="n">
+        <x:v>0.014017216318015335</x:v>
+      </x:c>
+      <x:c r="H6" s="21" t="n">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="I6" s="21" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J6" s="21"/>
+      <x:c r="K6" s="21"/>
+      <x:c r="L6" s="21"/>
+      <x:c r="M6" s="21"/>
+      <x:c r="N6" s="21"/>
+      <x:c r="O6" s="21"/>
+      <x:c r="P6" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>BB4652</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>UC4</x:v>
+      </x:c>
+      <x:c r="D7" s="21" t="str">
+        <x:v>UC</x:v>
+      </x:c>
+      <x:c r="E7" s="21" t="n">
+        <x:v>0.5980533100483266</x:v>
+      </x:c>
+      <x:c r="F7" s="21" t="n">
+        <x:v>0.6597357492065963</x:v>
+      </x:c>
+      <x:c r="G7" s="21" t="n">
+        <x:v>0.06168243915826965</x:v>
+      </x:c>
+      <x:c r="H7" s="21" t="n">
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="I7" s="21" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="J7" s="21"/>
+      <x:c r="K7" s="21"/>
+      <x:c r="L7" s="21"/>
+      <x:c r="M7" s="21"/>
+      <x:c r="N7" s="21"/>
+      <x:c r="O7" s="21"/>
+      <x:c r="P7" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21" t="str">
+        <x:v>donor</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>GI 4980</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>UC5</x:v>
+      </x:c>
+      <x:c r="D8" s="21" t="str">
+        <x:v>UC</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="n">
+        <x:v>0.5811378934524214</x:v>
+      </x:c>
+      <x:c r="F8" s="21" t="n">
+        <x:v>0.6144958892639544</x:v>
+      </x:c>
+      <x:c r="G8" s="21" t="n">
+        <x:v>0.03335799581153298</x:v>
+      </x:c>
+      <x:c r="H8" s="21" t="n">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="I8" s="21" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="J8" s="21"/>
+      <x:c r="K8" s="21"/>
+      <x:c r="L8" s="21"/>
+      <x:c r="M8" s="21"/>
+      <x:c r="N8" s="21"/>
+      <x:c r="O8" s="21"/>
+      <x:c r="P8" s="21" t="str">
+        <x:v>One donor; spots summarized within donor and not treated as independent replicates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="21" t="str">
+        <x:v>summary</x:v>
+      </x:c>
+      <x:c r="B9" s="21"/>
+      <x:c r="C9" s="21"/>
+      <x:c r="D9" s="21"/>
+      <x:c r="E9" s="21"/>
+      <x:c r="F9" s="21"/>
+      <x:c r="G9" s="21"/>
+      <x:c r="H9" s="21"/>
+      <x:c r="I9" s="21"/>
+      <x:c r="J9" s="21" t="n">
+        <x:v>0.02620254269391309</x:v>
+      </x:c>
+      <x:c r="K9" s="21" t="n">
+        <x:v>0.01399996188877057</x:v>
+      </x:c>
+      <x:c r="L9" s="21" t="n">
+        <x:v>0.040668972787999115</x:v>
+      </x:c>
+      <x:c r="M9" s="21" t="n">
+        <x:v>0.015625</x:v>
+      </x:c>
+      <x:c r="N9" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O9" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="P9" s="21" t="str">
+        <x:v>Donor-level two-sided exact paired sign-flip test; donor bootstrap 95% CI</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>